<commit_message>
Added most up to date workflow sampling
</commit_message>
<xml_diff>
--- a/Research/Workflow Analysis/Workflow_Analysis_Draft_5.xlsx
+++ b/Research/Workflow Analysis/Workflow_Analysis_Draft_5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marci/Desktop/Creative-Visual-Design-Accessibility-Tools/Research/Workflow Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57B17F78-7A21-E642-9CED-3CFB526E2EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBB1D44-BE4E-4540-8D0A-A537F6473C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17340" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TEMPLATE" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1320" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="326">
   <si>
     <t>Title</t>
   </si>
@@ -992,6 +992,39 @@
   </si>
   <si>
     <t>pan around in different directions</t>
+  </si>
+  <si>
+    <t>10_1</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=uz9tPsak9pM&amp;list=PLrJQSKQvgHS73G9sOhMhmWk-JoJZsyPiX</t>
+  </si>
+  <si>
+    <t>Design some social media templates with me! [Livestream Replay]</t>
+  </si>
+  <si>
+    <t>select assets on toolbar</t>
+  </si>
+  <si>
+    <t>scroll through assets</t>
+  </si>
+  <si>
+    <t>drag and drop asset</t>
+  </si>
+  <si>
+    <t>very small resizing</t>
+  </si>
+  <si>
+    <t>update colour using GUI</t>
+  </si>
+  <si>
+    <t>zoom out and in again</t>
+  </si>
+  <si>
+    <t>change design file e.g. navigating through figma interface to find new assets file</t>
+  </si>
+  <si>
+    <t>switch back to original design file</t>
   </si>
 </sst>
 </file>
@@ -7958,7 +7991,7 @@
     <col min="2" max="2" width="6.1640625" customWidth="1"/>
     <col min="3" max="3" width="7.33203125" customWidth="1"/>
     <col min="4" max="4" width="5.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="67.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="63.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="76.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33" customWidth="1"/>
     <col min="9" max="9" width="26.83203125" customWidth="1"/>
@@ -8044,23 +8077,23 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>270</v>
+        <v>317</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>288</v>
+        <v>316</v>
       </c>
       <c r="C2" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="D2" s="3">
-        <v>86.56</v>
+        <v>57</v>
       </c>
       <c r="E2" s="3">
-        <v>86.56</v>
+        <v>57.02</v>
       </c>
       <c r="F2" s="17"/>
       <c r="G2" s="17" t="s">
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="O2">
         <f t="shared" ref="O2:P33" si="0">(INT(D2)*60+(D2-INT(D2))*100)-(INT($D$2)*60+($D$2-INT($D$2))*100)</f>
@@ -8068,122 +8101,118 @@
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.0000000000004547</v>
       </c>
       <c r="Q2">
         <f t="shared" ref="Q2:Q58" si="1">P2-O2</f>
-        <v>0</v>
+        <v>2.0000000000004547</v>
       </c>
       <c r="R2" t="str">
         <f t="shared" ref="R2:R58" si="2">IF(Q2=0,"&lt;1 second","&lt;"&amp;(ROUND(Q2,2)+1)&amp;" seconds")</f>
-        <v>&lt;1 second</v>
+        <v>&lt;3 seconds</v>
       </c>
       <c r="S2">
         <f t="shared" ref="S2:S58" si="3">Q2+1</f>
-        <v>1</v>
+        <v>3.0000000000004547</v>
       </c>
       <c r="T2">
         <f t="shared" ref="T2:T58" si="4">Q2+0.5</f>
-        <v>0.5</v>
+        <v>2.5000000000004547</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D3" s="3">
-        <v>86.56</v>
+        <v>57.02</v>
       </c>
       <c r="E3" s="3">
-        <f>86.58</f>
-        <v>86.58</v>
+        <v>57.03</v>
       </c>
       <c r="F3" s="17"/>
       <c r="G3" s="17" t="s">
-        <v>147</v>
+        <v>32</v>
       </c>
       <c r="O3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.0000000000004547</v>
       </c>
       <c r="P3">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q3">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>0.99999999999954525</v>
       </c>
       <c r="R3" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;3 seconds</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S3">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>1.9999999999995453</v>
       </c>
       <c r="T3">
         <f t="shared" si="4"/>
-        <v>2.5</v>
+        <v>1.4999999999995453</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D4" s="3">
-        <v>86.59</v>
+        <v>57.04</v>
       </c>
       <c r="E4" s="3">
-        <f t="shared" ref="E4:E51" si="5">D4</f>
-        <v>86.59</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>290</v>
-      </c>
+        <v>57.05</v>
+      </c>
+      <c r="F4" s="17"/>
       <c r="G4" s="17" t="s">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="O4">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P4">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4.9999999999995453</v>
       </c>
       <c r="Q4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.99999999999954525</v>
       </c>
       <c r="R4" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>1.9999999999995453</v>
       </c>
       <c r="T4">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>1.4999999999995453</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D5" s="3">
-        <v>87.01</v>
+        <v>57.06</v>
       </c>
       <c r="E5" s="3">
-        <f t="shared" si="5"/>
-        <v>87.01</v>
+        <f t="shared" ref="E3:E58" si="5">D5</f>
+        <v>57.06</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>291</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>292</v>
+        <v>318</v>
+      </c>
+      <c r="G5" t="s">
+        <v>50</v>
       </c>
       <c r="O5">
         <f t="shared" si="0"/>
-        <v>5.0000000000009095</v>
+        <v>6</v>
       </c>
       <c r="P5">
         <f t="shared" si="0"/>
-        <v>5.0000000000009095</v>
+        <v>6</v>
       </c>
       <c r="Q5">
         <f t="shared" si="1"/>
@@ -8204,138 +8233,135 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D6" s="3">
-        <v>87.02</v>
+        <v>57.07</v>
       </c>
       <c r="E6" s="3">
-        <f t="shared" si="5"/>
-        <v>87.02</v>
+        <v>57.1</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>293</v>
+        <v>319</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>147</v>
+        <v>50</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="Q6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R6" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;4 seconds</v>
       </c>
       <c r="S6">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T6">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D7" s="3">
-        <v>87.04</v>
+        <v>57.1</v>
       </c>
       <c r="E7" s="3">
-        <f t="shared" si="5"/>
-        <v>87.04</v>
-      </c>
-      <c r="F7" s="17"/>
+        <v>57.11</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>320</v>
+      </c>
       <c r="G7" s="17" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="O7">
         <f t="shared" si="0"/>
-        <v>8.0000000000009095</v>
+        <v>10</v>
       </c>
       <c r="P7">
         <f t="shared" si="0"/>
-        <v>8.0000000000009095</v>
+        <v>11</v>
       </c>
       <c r="Q7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S7">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D8" s="3">
-        <v>87.04</v>
+        <v>57.11</v>
       </c>
       <c r="E8" s="3">
-        <f t="shared" si="5"/>
-        <v>87.04</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>161</v>
-      </c>
+        <v>57.12</v>
+      </c>
+      <c r="F8" s="17"/>
       <c r="G8" s="17" t="s">
-        <v>28</v>
+        <v>147</v>
       </c>
       <c r="O8">
         <f t="shared" si="0"/>
-        <v>8.0000000000009095</v>
+        <v>11</v>
       </c>
       <c r="P8">
         <f t="shared" si="0"/>
-        <v>8.0000000000009095</v>
+        <v>11.999999999999545</v>
       </c>
       <c r="Q8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.99999999999954525</v>
       </c>
       <c r="R8" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S8">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>1.9999999999995453</v>
       </c>
       <c r="T8">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>1.4999999999995453</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D9" s="3">
-        <v>87.04</v>
+        <v>57.12</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="5"/>
-        <v>87.04</v>
+        <v>57.12</v>
       </c>
       <c r="F9" s="17"/>
       <c r="G9" s="17" t="s">
-        <v>147</v>
+        <v>24</v>
       </c>
       <c r="O9">
         <f t="shared" si="0"/>
-        <v>8.0000000000009095</v>
+        <v>11.999999999999545</v>
       </c>
       <c r="P9">
         <f t="shared" si="0"/>
-        <v>8.0000000000009095</v>
+        <v>11.999999999999545</v>
       </c>
       <c r="Q9">
         <f t="shared" si="1"/>
@@ -8356,25 +8382,23 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D10" s="3">
-        <v>87.05</v>
+        <v>57.13</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="5"/>
-        <v>87.05</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>296</v>
-      </c>
+        <v>57.13</v>
+      </c>
+      <c r="F10" s="17"/>
       <c r="G10" s="17" t="s">
-        <v>152</v>
+        <v>185</v>
       </c>
       <c r="O10">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>13.000000000000455</v>
       </c>
       <c r="P10">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>13.000000000000455</v>
       </c>
       <c r="Q10">
         <f t="shared" si="1"/>
@@ -8395,23 +8419,23 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D11" s="3">
-        <v>87.05</v>
+        <v>57.15</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="5"/>
-        <v>87.05</v>
+        <v>57.15</v>
       </c>
       <c r="F11" s="17"/>
       <c r="G11" s="17" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="O11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="P11">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="Q11">
         <f t="shared" si="1"/>
@@ -8432,137 +8456,137 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D12" s="3">
-        <v>87.06</v>
+        <v>57.16</v>
       </c>
       <c r="E12" s="3">
-        <v>87.09</v>
+        <v>57.17</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>294</v>
+        <v>321</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>50</v>
+        <v>155</v>
       </c>
       <c r="O12">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>15.999999999999545</v>
       </c>
       <c r="P12">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q12">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>1.0000000000004547</v>
       </c>
       <c r="R12" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;4 seconds</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S12">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>2.0000000000004547</v>
       </c>
       <c r="T12">
         <f t="shared" si="4"/>
-        <v>3.5</v>
+        <v>1.5000000000004547</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D13" s="3">
-        <v>87.1</v>
+        <v>57.17</v>
       </c>
       <c r="E13" s="3">
-        <f t="shared" si="5"/>
-        <v>87.1</v>
-      </c>
-      <c r="F13" s="17"/>
+        <v>57.2</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>322</v>
+      </c>
       <c r="G13" s="17" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="O13">
         <f t="shared" si="0"/>
-        <v>13.999999999999091</v>
+        <v>17</v>
       </c>
       <c r="P13">
         <f t="shared" si="0"/>
-        <v>13.999999999999091</v>
+        <v>20.000000000000455</v>
       </c>
       <c r="Q13">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.0000000000004547</v>
       </c>
       <c r="R13" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;4 seconds</v>
       </c>
       <c r="S13">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>4.0000000000004547</v>
       </c>
       <c r="T13">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>3.5000000000004547</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D14" s="3">
-        <v>87.11</v>
+        <v>57.21</v>
       </c>
       <c r="E14" s="3">
-        <f t="shared" si="5"/>
-        <v>87.11</v>
-      </c>
-      <c r="F14" s="17" t="s">
-        <v>295</v>
-      </c>
+        <v>57.22</v>
+      </c>
+      <c r="F14" s="17"/>
       <c r="G14" s="17" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="O14">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="P14">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="Q14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S14">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D15" s="3">
-        <v>87.12</v>
+        <v>57.23</v>
       </c>
       <c r="E15" s="3">
         <f t="shared" si="5"/>
-        <v>87.12</v>
-      </c>
-      <c r="F15" s="17"/>
+        <v>57.23</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>161</v>
+      </c>
       <c r="G15" s="17" t="s">
-        <v>152</v>
+        <v>28</v>
       </c>
       <c r="O15">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>22.999999999999545</v>
       </c>
       <c r="P15">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>22.999999999999545</v>
       </c>
       <c r="Q15">
         <f t="shared" si="1"/>
@@ -8583,171 +8607,172 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D16" s="3">
-        <v>87.14</v>
+        <v>57.23</v>
       </c>
       <c r="E16" s="3">
-        <f t="shared" si="5"/>
-        <v>87.14</v>
+        <v>57.24</v>
       </c>
       <c r="F16" s="17"/>
       <c r="G16" s="17" t="s">
-        <v>147</v>
+        <v>34</v>
       </c>
       <c r="O16">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>22.999999999999545</v>
       </c>
       <c r="P16">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="Q16">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.0000000000004547</v>
       </c>
       <c r="R16" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S16">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2.0000000000004547</v>
       </c>
       <c r="T16">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>1.5000000000004547</v>
       </c>
     </row>
     <row r="17" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D17" s="3">
-        <v>87.15</v>
+        <v>57.25</v>
       </c>
       <c r="E17" s="3">
-        <f t="shared" si="5"/>
-        <v>87.15</v>
-      </c>
-      <c r="F17" s="17"/>
+        <v>57.26</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>323</v>
+      </c>
       <c r="G17" s="17" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="O17">
         <f t="shared" si="0"/>
-        <v>19.000000000000909</v>
+        <v>25</v>
       </c>
       <c r="P17">
         <f t="shared" si="0"/>
-        <v>19.000000000000909</v>
+        <v>26</v>
       </c>
       <c r="Q17">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;2 seconds</v>
       </c>
       <c r="S17">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T17">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="18" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D18" s="3">
-        <v>87.15</v>
+        <v>57.27</v>
       </c>
       <c r="E18" s="3">
-        <v>87.17</v>
-      </c>
-      <c r="F18" s="17"/>
+        <v>57.47</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>324</v>
+      </c>
       <c r="G18" s="17" t="s">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="O18">
         <f t="shared" si="0"/>
-        <v>19.000000000000909</v>
+        <v>27.000000000000455</v>
       </c>
       <c r="P18">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="Q18">
         <f t="shared" si="1"/>
-        <v>1.9999999999990905</v>
+        <v>19.999999999999545</v>
       </c>
       <c r="R18" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;3 seconds</v>
+        <v>&lt;21 seconds</v>
       </c>
       <c r="S18">
         <f t="shared" si="3"/>
-        <v>2.9999999999990905</v>
+        <v>20.999999999999545</v>
       </c>
       <c r="T18">
         <f t="shared" si="4"/>
-        <v>2.4999999999990905</v>
+        <v>20.499999999999545</v>
       </c>
     </row>
     <row r="19" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D19" s="3">
-        <v>87.17</v>
+        <v>57.51</v>
       </c>
       <c r="E19" s="3">
-        <v>87.18</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>297</v>
-      </c>
+        <f t="shared" si="5"/>
+        <v>57.51</v>
+      </c>
+      <c r="F19" s="17"/>
       <c r="G19" s="17" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="O19">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="P19">
         <f t="shared" si="0"/>
-        <v>22.000000000000909</v>
+        <v>51</v>
       </c>
       <c r="Q19">
         <f t="shared" si="1"/>
-        <v>1.0000000000009095</v>
+        <v>0</v>
       </c>
       <c r="R19" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
+        <v>&lt;1 second</v>
       </c>
       <c r="S19">
         <f t="shared" si="3"/>
-        <v>2.0000000000009095</v>
+        <v>1</v>
       </c>
       <c r="T19">
         <f t="shared" si="4"/>
-        <v>1.5000000000009095</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="20" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D20" s="3">
-        <v>87.19</v>
+        <v>57.51</v>
       </c>
       <c r="E20" s="3">
         <f t="shared" si="5"/>
-        <v>87.19</v>
+        <v>57.51</v>
       </c>
       <c r="F20" s="17"/>
       <c r="G20" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="O20">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="P20">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="Q20">
         <f t="shared" si="1"/>
@@ -8768,23 +8793,23 @@
     </row>
     <row r="21" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D21" s="3">
-        <v>87.2</v>
+        <v>57.51</v>
       </c>
       <c r="E21" s="3">
         <f t="shared" si="5"/>
-        <v>87.2</v>
+        <v>57.51</v>
       </c>
       <c r="F21" s="17"/>
       <c r="G21" s="17" t="s">
-        <v>28</v>
+        <v>304</v>
       </c>
       <c r="O21">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="P21">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="Q21">
         <f t="shared" si="1"/>
@@ -8805,60 +8830,61 @@
     </row>
     <row r="22" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D22" s="3">
-        <v>87.2</v>
+        <v>57.53</v>
       </c>
       <c r="E22" s="3">
-        <f t="shared" si="5"/>
-        <v>87.2</v>
-      </c>
-      <c r="F22" s="17"/>
+        <v>57.56</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>325</v>
+      </c>
       <c r="G22" s="17" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="O22">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="P22">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Q22">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R22" t="str">
         <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
+        <v>&lt;4 seconds</v>
       </c>
       <c r="S22">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T22">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="23" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D23" s="3">
-        <v>87.2</v>
+        <v>57.57</v>
       </c>
       <c r="E23" s="3">
         <f t="shared" si="5"/>
-        <v>87.2</v>
+        <v>57.57</v>
       </c>
       <c r="F23" s="17"/>
       <c r="G23" s="17" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="O23">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="P23">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="Q23">
         <f t="shared" si="1"/>
@@ -8879,25 +8905,23 @@
     </row>
     <row r="24" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D24" s="3">
-        <v>87.21</v>
+        <v>58.01</v>
       </c>
       <c r="E24" s="3">
         <f t="shared" si="5"/>
-        <v>87.21</v>
-      </c>
-      <c r="F24" s="17" t="s">
-        <v>290</v>
-      </c>
+        <v>58.01</v>
+      </c>
+      <c r="F24" s="17"/>
       <c r="G24" s="17" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="O24">
         <f t="shared" si="0"/>
-        <v>24.999999999999091</v>
+        <v>61</v>
       </c>
       <c r="P24">
         <f t="shared" si="0"/>
-        <v>24.999999999999091</v>
+        <v>61</v>
       </c>
       <c r="Q24">
         <f t="shared" si="1"/>
@@ -8918,23 +8942,23 @@
     </row>
     <row r="25" spans="4:20" x14ac:dyDescent="0.2">
       <c r="D25" s="3">
-        <v>87.22</v>
+        <v>58.02</v>
       </c>
       <c r="E25" s="3">
         <f t="shared" si="5"/>
-        <v>87.22</v>
+        <v>58.02</v>
       </c>
       <c r="F25" s="17"/>
-      <c r="G25" s="18" t="s">
-        <v>292</v>
+      <c r="G25" s="17" t="s">
+        <v>282</v>
       </c>
       <c r="O25">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>62.000000000000455</v>
       </c>
       <c r="P25">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>62.000000000000455</v>
       </c>
       <c r="Q25">
         <f t="shared" si="1"/>
@@ -8954,1246 +8978,173 @@
       </c>
     </row>
     <row r="26" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D26" s="3">
-        <v>87.22</v>
-      </c>
-      <c r="E26" s="3">
-        <v>87.23</v>
-      </c>
-      <c r="F26" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="G26" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="O26">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="P26">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="Q26">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R26" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S26">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="T26">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
-      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
     </row>
     <row r="27" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D27" s="3">
-        <v>87.23</v>
-      </c>
-      <c r="E27" s="3">
-        <f t="shared" si="5"/>
-        <v>87.23</v>
-      </c>
+      <c r="E27" s="3"/>
       <c r="F27" s="17"/>
-      <c r="G27" s="18" t="s">
-        <v>292</v>
-      </c>
-      <c r="O27">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="P27">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="Q27">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R27" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S27">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T27">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
+      <c r="G27" s="17"/>
     </row>
     <row r="28" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D28" s="3">
-        <v>87.23</v>
-      </c>
-      <c r="E28" s="3">
-        <f t="shared" si="5"/>
-        <v>87.23</v>
-      </c>
-      <c r="F28" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="G28" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="O28">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="P28">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="Q28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R28" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S28">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T28">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
     </row>
     <row r="29" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D29" s="3">
-        <v>87.24</v>
-      </c>
-      <c r="E29" s="3">
-        <f t="shared" si="5"/>
-        <v>87.24</v>
-      </c>
+      <c r="E29" s="3"/>
       <c r="F29" s="17"/>
-      <c r="G29" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="O29">
-        <f t="shared" si="0"/>
-        <v>27.999999999999091</v>
-      </c>
-      <c r="P29">
-        <f t="shared" si="0"/>
-        <v>27.999999999999091</v>
-      </c>
-      <c r="Q29">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R29" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S29">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T29">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
+      <c r="G29" s="17"/>
     </row>
     <row r="30" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D30" s="3">
-        <v>87.25</v>
-      </c>
-      <c r="E30" s="3">
-        <f t="shared" si="5"/>
-        <v>87.25</v>
-      </c>
-      <c r="F30" s="17" t="s">
-        <v>298</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="O30">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="P30">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="Q30">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R30" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S30">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T30">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
+      <c r="E30" s="3"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
     </row>
     <row r="31" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D31" s="3">
-        <v>87.25</v>
-      </c>
-      <c r="E31" s="3">
-        <f t="shared" si="5"/>
-        <v>87.25</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>299</v>
-      </c>
-      <c r="G31" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="O31">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="P31">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="Q31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R31" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S31">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T31">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
+      <c r="E31" s="3"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
     </row>
     <row r="32" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D32" s="3">
-        <v>87.26</v>
-      </c>
-      <c r="E32" s="3">
-        <f t="shared" si="5"/>
-        <v>87.26</v>
-      </c>
+      <c r="E32" s="3"/>
       <c r="F32" s="17"/>
-      <c r="G32" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="O32">
-        <f t="shared" si="0"/>
-        <v>30.000000000000909</v>
-      </c>
-      <c r="P32">
-        <f t="shared" si="0"/>
-        <v>30.000000000000909</v>
-      </c>
-      <c r="Q32">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R32" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S32">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T32">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="33" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D33" s="3">
-        <v>87.3</v>
-      </c>
-      <c r="E33" s="3">
-        <f t="shared" si="5"/>
-        <v>87.3</v>
-      </c>
-      <c r="F33" s="17" t="s">
-        <v>290</v>
-      </c>
-      <c r="G33" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="O33">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="P33">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="Q33">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R33" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S33">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T33">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="34" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D34" s="3">
-        <v>87.31</v>
-      </c>
-      <c r="E34" s="3">
-        <f t="shared" si="5"/>
-        <v>87.31</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>300</v>
-      </c>
-      <c r="G34" s="18" t="s">
-        <v>301</v>
-      </c>
-      <c r="O34">
-        <f t="shared" ref="O34:P66" si="6">(INT(D34)*60+(D34-INT(D34))*100)-(INT($D$2)*60+($D$2-INT($D$2))*100)</f>
-        <v>35</v>
-      </c>
-      <c r="P34">
-        <f t="shared" si="6"/>
-        <v>35</v>
-      </c>
-      <c r="Q34">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R34" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S34">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T34">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="35" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D35" s="3">
-        <v>87.33</v>
-      </c>
-      <c r="E35" s="3">
-        <f t="shared" si="5"/>
-        <v>87.33</v>
-      </c>
+      <c r="G32" s="17"/>
+    </row>
+    <row r="33" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E33" s="3"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+    </row>
+    <row r="34" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E34" s="3"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+    </row>
+    <row r="35" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E35" s="3"/>
       <c r="F35" s="17"/>
-      <c r="G35" s="18" t="s">
-        <v>292</v>
-      </c>
-      <c r="O35">
-        <f t="shared" si="6"/>
-        <v>37</v>
-      </c>
-      <c r="P35">
-        <f t="shared" si="6"/>
-        <v>37</v>
-      </c>
-      <c r="Q35">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R35" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S35">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T35">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="36" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D36" s="3">
-        <v>87.33</v>
-      </c>
-      <c r="E36" s="3">
-        <v>87.34</v>
-      </c>
-      <c r="F36" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="G36" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="O36">
-        <f t="shared" si="6"/>
-        <v>37</v>
-      </c>
-      <c r="P36">
-        <f t="shared" si="6"/>
-        <v>38</v>
-      </c>
-      <c r="Q36">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R36" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S36">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="T36">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="37" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D37" s="3">
-        <v>87.34</v>
-      </c>
-      <c r="E37" s="3">
-        <f t="shared" si="5"/>
-        <v>87.34</v>
-      </c>
+      <c r="G35" s="17"/>
+    </row>
+    <row r="36" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E36" s="3"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+    </row>
+    <row r="37" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E37" s="3"/>
       <c r="F37" s="17"/>
-      <c r="G37" s="18" t="s">
-        <v>292</v>
-      </c>
-      <c r="O37">
-        <f t="shared" si="6"/>
-        <v>38</v>
-      </c>
-      <c r="P37">
-        <f t="shared" si="6"/>
-        <v>38</v>
-      </c>
-      <c r="Q37">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R37" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S37">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T37">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="38" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D38" s="3">
-        <v>87.34</v>
-      </c>
-      <c r="E38" s="3">
-        <v>87.37</v>
-      </c>
+      <c r="G37" s="17"/>
+    </row>
+    <row r="38" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E38" s="3"/>
       <c r="F38" s="17"/>
-      <c r="G38" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="O38">
-        <f t="shared" si="6"/>
-        <v>38</v>
-      </c>
-      <c r="P38">
-        <f t="shared" si="6"/>
-        <v>41</v>
-      </c>
-      <c r="Q38">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="R38" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;4 seconds</v>
-      </c>
-      <c r="S38">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="T38">
-        <f t="shared" si="4"/>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="39" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D39" s="3">
-        <v>87.37</v>
-      </c>
-      <c r="E39" s="3">
-        <f t="shared" si="5"/>
-        <v>87.37</v>
-      </c>
+      <c r="G38" s="17"/>
+    </row>
+    <row r="39" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E39" s="3"/>
       <c r="F39" s="17"/>
-      <c r="G39" s="18" t="s">
-        <v>302</v>
-      </c>
-      <c r="O39">
-        <f t="shared" si="6"/>
-        <v>41</v>
-      </c>
-      <c r="P39">
-        <f t="shared" si="6"/>
-        <v>41</v>
-      </c>
-      <c r="Q39">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R39" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S39">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T39">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="40" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D40" s="3">
-        <v>87.38</v>
-      </c>
-      <c r="E40" s="3">
-        <v>87.39</v>
-      </c>
-      <c r="F40" s="17" t="s">
-        <v>303</v>
-      </c>
-      <c r="G40" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="O40">
-        <f t="shared" si="6"/>
-        <v>42</v>
-      </c>
-      <c r="P40">
-        <f t="shared" si="6"/>
-        <v>43</v>
-      </c>
-      <c r="Q40">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R40" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S40">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="T40">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="41" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D41" s="3">
-        <v>87.39</v>
-      </c>
-      <c r="E41" s="3">
-        <f t="shared" si="5"/>
-        <v>87.39</v>
-      </c>
+      <c r="G39" s="17"/>
+    </row>
+    <row r="40" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E40" s="3"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+    </row>
+    <row r="41" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E41" s="3"/>
       <c r="F41" s="17"/>
-      <c r="G41" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="O41">
-        <f t="shared" si="6"/>
-        <v>43</v>
-      </c>
-      <c r="P41">
-        <f t="shared" si="6"/>
-        <v>43</v>
-      </c>
-      <c r="Q41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R41" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S41">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T41">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="42" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D42" s="3">
-        <v>87.4</v>
-      </c>
-      <c r="E42" s="3">
-        <f t="shared" si="5"/>
-        <v>87.4</v>
-      </c>
-      <c r="G42" t="s">
-        <v>26</v>
-      </c>
-      <c r="O42">
-        <f t="shared" si="6"/>
-        <v>44.000000000000909</v>
-      </c>
-      <c r="P42">
-        <f t="shared" si="6"/>
-        <v>44.000000000000909</v>
-      </c>
-      <c r="Q42">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R42" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S42">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T42">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="43" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D43" s="3">
-        <v>87.4</v>
-      </c>
-      <c r="E43" s="3">
-        <f t="shared" si="5"/>
-        <v>87.4</v>
-      </c>
-      <c r="F43" t="s">
-        <v>161</v>
-      </c>
-      <c r="G43" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="O43">
-        <f t="shared" si="6"/>
-        <v>44.000000000000909</v>
-      </c>
-      <c r="P43">
-        <f t="shared" si="6"/>
-        <v>44.000000000000909</v>
-      </c>
-      <c r="Q43">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R43" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S43">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T43">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="44" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D44" s="3">
-        <v>87.42</v>
-      </c>
-      <c r="E44" s="3">
-        <f t="shared" si="5"/>
-        <v>87.42</v>
-      </c>
-      <c r="F44" t="s">
-        <v>161</v>
-      </c>
-      <c r="G44" t="s">
-        <v>28</v>
-      </c>
-      <c r="O44">
-        <f t="shared" si="6"/>
-        <v>46</v>
-      </c>
-      <c r="P44">
-        <f t="shared" si="6"/>
-        <v>46</v>
-      </c>
-      <c r="Q44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R44" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S44">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T44">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="45" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D45" s="3">
-        <v>87.42</v>
-      </c>
-      <c r="E45" s="3">
-        <v>87.43</v>
-      </c>
-      <c r="F45" t="s">
-        <v>237</v>
-      </c>
-      <c r="G45" t="s">
-        <v>152</v>
-      </c>
-      <c r="O45">
-        <f t="shared" si="6"/>
-        <v>46</v>
-      </c>
-      <c r="P45">
-        <f t="shared" si="6"/>
-        <v>47.000000000000909</v>
-      </c>
-      <c r="Q45">
-        <f t="shared" si="1"/>
-        <v>1.0000000000009095</v>
-      </c>
-      <c r="R45" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S45">
-        <f t="shared" si="3"/>
-        <v>2.0000000000009095</v>
-      </c>
-      <c r="T45">
-        <f t="shared" si="4"/>
-        <v>1.5000000000009095</v>
-      </c>
-    </row>
-    <row r="46" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D46" s="3">
-        <v>87.43</v>
-      </c>
-      <c r="E46" s="3">
-        <f t="shared" si="5"/>
-        <v>87.43</v>
-      </c>
-      <c r="G46" t="s">
-        <v>153</v>
-      </c>
-      <c r="O46">
-        <f t="shared" si="6"/>
-        <v>47.000000000000909</v>
-      </c>
-      <c r="P46">
-        <f t="shared" si="6"/>
-        <v>47.000000000000909</v>
-      </c>
-      <c r="Q46">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R46" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S46">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T46">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="47" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D47" s="3">
-        <v>87.43</v>
-      </c>
-      <c r="E47" s="3">
-        <v>87.44</v>
-      </c>
-      <c r="G47" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="O47">
-        <f t="shared" si="6"/>
-        <v>47.000000000000909</v>
-      </c>
-      <c r="P47">
-        <f t="shared" si="6"/>
-        <v>48</v>
-      </c>
-      <c r="Q47">
-        <f t="shared" si="1"/>
-        <v>0.99999999999909051</v>
-      </c>
-      <c r="R47" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S47">
-        <f t="shared" si="3"/>
-        <v>1.9999999999990905</v>
-      </c>
-      <c r="T47">
-        <f t="shared" si="4"/>
-        <v>1.4999999999990905</v>
-      </c>
-    </row>
-    <row r="48" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D48" s="3">
-        <v>87.45</v>
-      </c>
-      <c r="E48" s="3">
-        <f t="shared" si="5"/>
-        <v>87.45</v>
-      </c>
-      <c r="G48" t="s">
-        <v>24</v>
-      </c>
-      <c r="O48">
-        <f t="shared" si="6"/>
-        <v>49</v>
-      </c>
-      <c r="P48">
-        <f t="shared" si="6"/>
-        <v>49</v>
-      </c>
-      <c r="Q48">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R48" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S48">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T48">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="49" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D49" s="3">
-        <v>87.46</v>
-      </c>
-      <c r="E49" s="3">
-        <v>87.46</v>
-      </c>
-      <c r="G49" t="s">
-        <v>26</v>
-      </c>
-      <c r="O49">
-        <f t="shared" si="6"/>
-        <v>49.999999999999091</v>
-      </c>
-      <c r="P49">
-        <f t="shared" si="6"/>
-        <v>49.999999999999091</v>
-      </c>
-      <c r="Q49">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R49" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S49">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T49">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="50" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D50" s="3">
-        <v>87.46</v>
-      </c>
-      <c r="E50" s="3">
-        <f t="shared" si="5"/>
-        <v>87.46</v>
-      </c>
-      <c r="F50" t="s">
-        <v>161</v>
-      </c>
-      <c r="G50" t="s">
-        <v>28</v>
-      </c>
-      <c r="O50">
-        <f t="shared" si="6"/>
-        <v>49.999999999999091</v>
-      </c>
-      <c r="P50">
-        <f t="shared" si="6"/>
-        <v>49.999999999999091</v>
-      </c>
-      <c r="Q50">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R50" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S50">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T50">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="51" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D51" s="3">
-        <v>87.46</v>
-      </c>
-      <c r="E51" s="3">
-        <f t="shared" si="5"/>
-        <v>87.46</v>
-      </c>
-      <c r="G51" t="s">
-        <v>153</v>
-      </c>
-      <c r="O51">
-        <f t="shared" si="6"/>
-        <v>49.999999999999091</v>
-      </c>
-      <c r="P51">
-        <f t="shared" si="6"/>
-        <v>49.999999999999091</v>
-      </c>
-      <c r="Q51">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R51" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S51">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T51">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="52" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D52" s="3">
-        <v>87.47</v>
-      </c>
-      <c r="E52" s="3">
-        <v>87.48</v>
-      </c>
-      <c r="F52" t="s">
-        <v>305</v>
-      </c>
-      <c r="G52" t="s">
-        <v>147</v>
-      </c>
-      <c r="O52">
-        <f t="shared" si="6"/>
-        <v>51</v>
-      </c>
-      <c r="P52">
-        <f t="shared" si="6"/>
-        <v>52</v>
-      </c>
-      <c r="Q52">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R52" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S52">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="T52">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="53" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D53" s="3">
-        <v>87.47</v>
-      </c>
-      <c r="E53" s="3">
-        <v>87.48</v>
-      </c>
-      <c r="G53" t="s">
-        <v>149</v>
-      </c>
-      <c r="O53">
-        <f t="shared" si="6"/>
-        <v>51</v>
-      </c>
-      <c r="P53">
-        <f t="shared" si="6"/>
-        <v>52</v>
-      </c>
-      <c r="Q53">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R53" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S53">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="T53">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="54" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D54" s="3">
-        <v>87.5</v>
-      </c>
-      <c r="E54" s="3">
-        <f>D54</f>
-        <v>87.5</v>
-      </c>
-      <c r="G54" t="s">
-        <v>24</v>
-      </c>
-      <c r="O54">
-        <f t="shared" si="6"/>
-        <v>54</v>
-      </c>
-      <c r="P54">
-        <f t="shared" si="6"/>
-        <v>54</v>
-      </c>
-      <c r="Q54">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R54" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;1 second</v>
-      </c>
-      <c r="S54">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="T54">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="55" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D55" s="3">
-        <v>87.51</v>
-      </c>
-      <c r="E55" s="3">
-        <v>87.52</v>
-      </c>
-      <c r="G55" s="18" t="s">
-        <v>306</v>
-      </c>
-      <c r="O55">
-        <f t="shared" si="6"/>
-        <v>55.000000000000909</v>
-      </c>
-      <c r="P55">
-        <f t="shared" si="6"/>
-        <v>56</v>
-      </c>
-      <c r="Q55">
-        <f t="shared" si="1"/>
-        <v>0.99999999999909051</v>
-      </c>
-      <c r="R55" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S55">
-        <f t="shared" si="3"/>
-        <v>1.9999999999990905</v>
-      </c>
-      <c r="T55">
-        <f t="shared" si="4"/>
-        <v>1.4999999999990905</v>
-      </c>
-    </row>
-    <row r="56" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D56" s="3">
-        <v>87.52</v>
-      </c>
-      <c r="E56" s="3">
-        <v>87.54</v>
-      </c>
-      <c r="F56" t="s">
-        <v>307</v>
-      </c>
-      <c r="G56" t="s">
-        <v>50</v>
-      </c>
-      <c r="O56">
-        <f t="shared" si="6"/>
-        <v>56</v>
-      </c>
-      <c r="P56">
-        <f t="shared" si="6"/>
-        <v>58.000000000000909</v>
-      </c>
-      <c r="Q56">
-        <f t="shared" si="1"/>
-        <v>2.0000000000009095</v>
-      </c>
-      <c r="R56" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;3 seconds</v>
-      </c>
-      <c r="S56">
-        <f t="shared" si="3"/>
-        <v>3.0000000000009095</v>
-      </c>
-      <c r="T56">
-        <f t="shared" si="4"/>
-        <v>2.5000000000009095</v>
-      </c>
-    </row>
-    <row r="57" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D57" s="3">
-        <v>87.54</v>
-      </c>
-      <c r="E57" s="3">
-        <v>87.55</v>
-      </c>
-      <c r="G57" t="s">
-        <v>155</v>
-      </c>
-      <c r="O57">
-        <f t="shared" si="6"/>
-        <v>58.000000000000909</v>
-      </c>
-      <c r="P57">
-        <f t="shared" si="6"/>
-        <v>59</v>
-      </c>
-      <c r="Q57">
-        <f t="shared" si="1"/>
-        <v>0.99999999999909051</v>
-      </c>
-      <c r="R57" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;2 seconds</v>
-      </c>
-      <c r="S57">
-        <f t="shared" si="3"/>
-        <v>1.9999999999990905</v>
-      </c>
-      <c r="T57">
-        <f t="shared" si="4"/>
-        <v>1.4999999999990905</v>
-      </c>
-    </row>
-    <row r="58" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="D58" s="3">
-        <v>87.55</v>
-      </c>
-      <c r="E58" s="3">
-        <v>87.58</v>
-      </c>
-      <c r="G58" t="s">
-        <v>66</v>
-      </c>
-      <c r="O58">
-        <f t="shared" si="6"/>
-        <v>59</v>
-      </c>
-      <c r="P58">
-        <f t="shared" si="6"/>
-        <v>62</v>
-      </c>
-      <c r="Q58">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="R58" t="str">
-        <f t="shared" si="2"/>
-        <v>&lt;4 seconds</v>
-      </c>
-      <c r="S58">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="T58">
-        <f t="shared" si="4"/>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="59" spans="4:20" x14ac:dyDescent="0.2">
+      <c r="G41" s="17"/>
+    </row>
+    <row r="42" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E42" s="3"/>
+      <c r="G42" s="17"/>
+    </row>
+    <row r="43" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E43" s="3"/>
+      <c r="G43" s="17"/>
+    </row>
+    <row r="44" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E44" s="3"/>
+      <c r="G44" s="17"/>
+    </row>
+    <row r="45" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E45" s="3"/>
+      <c r="G45" s="17"/>
+    </row>
+    <row r="46" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E46" s="3"/>
+      <c r="G46" s="17"/>
+    </row>
+    <row r="47" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E47" s="3"/>
+      <c r="G47" s="17"/>
+    </row>
+    <row r="48" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E48" s="3"/>
+      <c r="G48" s="17"/>
+    </row>
+    <row r="49" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E49" s="3"/>
+      <c r="G49" s="17"/>
+    </row>
+    <row r="50" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E50" s="3"/>
+      <c r="G50" s="17"/>
+    </row>
+    <row r="51" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E51" s="3"/>
+      <c r="G51" s="17"/>
+    </row>
+    <row r="52" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E52" s="3"/>
+      <c r="G52" s="17"/>
+    </row>
+    <row r="53" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E53" s="3"/>
+      <c r="G53" s="17"/>
+    </row>
+    <row r="54" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E54" s="3"/>
+      <c r="G54" s="17"/>
+    </row>
+    <row r="55" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E55" s="3"/>
+      <c r="G55" s="17"/>
+    </row>
+    <row r="56" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E56" s="3"/>
+      <c r="G56" s="17"/>
+    </row>
+    <row r="57" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E57" s="3"/>
+      <c r="G57" s="17"/>
+    </row>
+    <row r="58" spans="5:7" x14ac:dyDescent="0.2">
+      <c r="E58" s="3"/>
+      <c r="G58" s="17"/>
+    </row>
+    <row r="59" spans="5:7" x14ac:dyDescent="0.2">
       <c r="E59" s="3"/>
-    </row>
-    <row r="60" spans="4:20" x14ac:dyDescent="0.2">
+      <c r="G59" s="17"/>
+    </row>
+    <row r="60" spans="5:7" x14ac:dyDescent="0.2">
       <c r="E60" s="3"/>
-    </row>
-    <row r="61" spans="4:20" x14ac:dyDescent="0.2">
+      <c r="G60" s="17"/>
+    </row>
+    <row r="61" spans="5:7" x14ac:dyDescent="0.2">
       <c r="E61" s="3"/>
-    </row>
-    <row r="62" spans="4:20" x14ac:dyDescent="0.2">
+      <c r="G61" s="17"/>
+    </row>
+    <row r="62" spans="5:7" x14ac:dyDescent="0.2">
       <c r="E62" s="3"/>
-    </row>
-    <row r="63" spans="4:20" x14ac:dyDescent="0.2">
+      <c r="G62" s="17"/>
+    </row>
+    <row r="63" spans="5:7" x14ac:dyDescent="0.2">
       <c r="E63" s="3"/>
     </row>
-    <row r="64" spans="4:20" x14ac:dyDescent="0.2">
+    <row r="64" spans="5:7" x14ac:dyDescent="0.2">
       <c r="E64" s="3"/>
     </row>
     <row r="65" spans="5:5" x14ac:dyDescent="0.2">
@@ -10249,7 +9200,7 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Please select a valid value from the list." sqref="G5 G39 G34" xr:uid="{B81AE3E2-B42B-264F-9B78-A9E7E223A592}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Please select a valid value from the list." sqref="G34 G39" xr:uid="{B81AE3E2-B42B-264F-9B78-A9E7E223A592}">
       <formula1>$A$2:$A$1001</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Please select a valid value from the list." sqref="M2:M1001" xr:uid="{1C40B2E5-0D5E-1440-92A3-C6C9E6BFB897}">
@@ -10826,7 +9777,7 @@
     <col min="7" max="7" width="78" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33" customWidth="1"/>
     <col min="9" max="9" width="26.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="14.33203125" customWidth="1"/>
     <col min="13" max="13" width="8.1640625" customWidth="1"/>
@@ -10930,7 +9881,9 @@
       <c r="I2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="J2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="K2" s="4" t="s">
         <v>47</v>
       </c>
@@ -10985,7 +9938,9 @@
       <c r="I3" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="8"/>
+      <c r="J3" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="K3" s="8" t="s">
         <v>52</v>
       </c>
@@ -11040,7 +9995,9 @@
       <c r="I4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="J4" s="4"/>
+      <c r="J4" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="K4" s="8" t="s">
         <v>54</v>
       </c>
@@ -11091,7 +10048,9 @@
       <c r="I5" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="J5" s="13"/>
+      <c r="J5" s="8" t="s">
+        <v>56</v>
+      </c>
       <c r="K5" s="8" t="s">
         <v>52</v>
       </c>
@@ -11144,7 +10103,9 @@
       <c r="I6" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="J6" s="8"/>
+      <c r="J6" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="K6" s="8" t="s">
         <v>61</v>
       </c>
@@ -11196,7 +10157,9 @@
       <c r="I7" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="J7" s="8"/>
+      <c r="J7" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="K7" s="8" t="s">
         <v>52</v>
       </c>
@@ -11250,7 +10213,9 @@
       <c r="I8" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="8"/>
+      <c r="J8" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="K8" s="8" t="s">
         <v>64</v>
       </c>
@@ -11305,7 +10270,9 @@
       <c r="I9" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J9" s="8"/>
+      <c r="J9" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="K9" s="8" t="s">
         <v>52</v>
       </c>
@@ -11355,7 +10322,9 @@
       <c r="I10" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J10" s="8"/>
+      <c r="J10" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="K10" s="8" t="s">
         <v>61</v>
       </c>
@@ -11407,7 +10376,9 @@
       <c r="I11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="J11" s="8"/>
+      <c r="J11" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="K11" s="8" t="s">
         <v>52</v>
       </c>
@@ -11462,7 +10433,9 @@
       <c r="I12" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="J12" s="8"/>
+      <c r="J12" s="8" t="s">
+        <v>73</v>
+      </c>
       <c r="K12" s="8" t="s">
         <v>61</v>
       </c>
@@ -11513,7 +10486,9 @@
       <c r="I13" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J13" s="8"/>
+      <c r="J13" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="K13" s="8" t="s">
         <v>52</v>
       </c>
@@ -11564,7 +10539,9 @@
       <c r="I14" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J14" s="8"/>
+      <c r="J14" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K14" s="8" t="s">
         <v>52</v>
       </c>
@@ -11615,7 +10592,9 @@
       <c r="I15" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="J15" s="8"/>
+      <c r="J15" s="8" t="s">
+        <v>77</v>
+      </c>
       <c r="K15" s="8" t="s">
         <v>61</v>
       </c>
@@ -11666,7 +10645,9 @@
       <c r="I16" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="J16" s="8"/>
+      <c r="J16" s="8" t="s">
+        <v>78</v>
+      </c>
       <c r="K16" s="8" t="s">
         <v>64</v>
       </c>
@@ -11720,7 +10701,9 @@
       <c r="I17" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J17" s="8"/>
+      <c r="J17" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K17" s="8" t="s">
         <v>52</v>
       </c>
@@ -11773,7 +10756,9 @@
       <c r="I18" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J18" s="8"/>
+      <c r="J18" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K18" s="8" t="s">
         <v>52</v>
       </c>
@@ -11871,7 +10856,9 @@
       <c r="I20" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="J20" s="8"/>
+      <c r="J20" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="K20" s="8" t="s">
         <v>64</v>
       </c>
@@ -11925,7 +10912,9 @@
       <c r="I21" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J21" s="8"/>
+      <c r="J21" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K21" s="8" t="s">
         <v>52</v>
       </c>
@@ -11977,7 +10966,9 @@
       <c r="I22" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J22" s="8"/>
+      <c r="J22" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="K22" s="8" t="s">
         <v>64</v>
       </c>
@@ -12032,7 +11023,9 @@
       <c r="I23" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J23" s="8"/>
+      <c r="J23" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K23" s="8" t="s">
         <v>83</v>
       </c>
@@ -12082,7 +11075,9 @@
       <c r="I24" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J24" s="8"/>
+      <c r="J24" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="K24" s="8" t="s">
         <v>64</v>
       </c>
@@ -12137,7 +11132,9 @@
       <c r="I25" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J25" s="8"/>
+      <c r="J25" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="K25" s="8" t="s">
         <v>54</v>
       </c>
@@ -12188,7 +11185,9 @@
       <c r="I26" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J26" s="8"/>
+      <c r="J26" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K26" s="8" t="s">
         <v>52</v>
       </c>
@@ -12238,7 +11237,9 @@
       <c r="I27" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="J27" s="8"/>
+      <c r="J27" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="K27" s="8" t="s">
         <v>61</v>
       </c>
@@ -12289,7 +11290,9 @@
       <c r="I28" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J28" s="8"/>
+      <c r="J28" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K28" s="8" t="s">
         <v>52</v>
       </c>
@@ -12339,7 +11342,9 @@
       <c r="I29" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="J29" s="8"/>
+      <c r="J29" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="K29" s="8" t="s">
         <v>61</v>
       </c>
@@ -12390,7 +11395,9 @@
       <c r="I30" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J30" s="8"/>
+      <c r="J30" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K30" s="8" t="s">
         <v>52</v>
       </c>
@@ -12441,7 +11448,9 @@
       <c r="I31" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J31" s="8"/>
+      <c r="J31" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="K31" s="8" t="s">
         <v>47</v>
       </c>
@@ -12492,7 +11501,9 @@
       <c r="I32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J32" s="8"/>
+      <c r="J32" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K32" s="8" t="s">
         <v>52</v>
       </c>
@@ -12542,7 +11553,9 @@
       <c r="I33" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J33" s="8"/>
+      <c r="J33" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="K33" s="8" t="s">
         <v>61</v>
       </c>
@@ -12593,7 +11606,9 @@
       <c r="I34" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J34" s="8"/>
+      <c r="J34" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K34" s="8" t="s">
         <v>52</v>
       </c>
@@ -12644,7 +11659,9 @@
       <c r="I35" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="J35" s="8"/>
+      <c r="J35" s="8" t="s">
+        <v>86</v>
+      </c>
       <c r="K35" s="8" t="s">
         <v>52</v>
       </c>
@@ -12699,7 +11716,9 @@
       <c r="I36" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J36" s="8"/>
+      <c r="J36" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="K36" s="8" t="s">
         <v>52</v>
       </c>
@@ -12753,7 +11772,9 @@
       <c r="I37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J37" s="8"/>
+      <c r="J37" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="K37" s="8" t="s">
         <v>47</v>
       </c>
@@ -12804,7 +11825,9 @@
       <c r="I38" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="J38" s="8"/>
+      <c r="J38" s="8" t="s">
+        <v>90</v>
+      </c>
       <c r="K38" s="8" t="s">
         <v>52</v>
       </c>
@@ -12856,7 +11879,9 @@
       <c r="I39" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="J39" s="8"/>
+      <c r="J39" s="8" t="s">
+        <v>92</v>
+      </c>
       <c r="K39" s="8" t="s">
         <v>52</v>
       </c>
@@ -12910,7 +11935,9 @@
       <c r="I40" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J40" s="8"/>
+      <c r="J40" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="K40" s="8" t="s">
         <v>52</v>
       </c>
@@ -12964,7 +11991,9 @@
       <c r="I41" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J41" s="8"/>
+      <c r="J41" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="K41" s="8" t="s">
         <v>52</v>
       </c>
@@ -13015,7 +12044,9 @@
       <c r="I42" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J42" s="8"/>
+      <c r="J42" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K42" s="8" t="s">
         <v>52</v>
       </c>
@@ -13066,7 +12097,9 @@
       <c r="I43" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="J43" s="8"/>
+      <c r="J43" s="8" t="s">
+        <v>77</v>
+      </c>
       <c r="K43" s="8" t="s">
         <v>61</v>
       </c>
@@ -13116,7 +12149,9 @@
       <c r="I44" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="J44" s="8"/>
+      <c r="J44" s="8" t="s">
+        <v>78</v>
+      </c>
       <c r="K44" s="8" t="s">
         <v>64</v>
       </c>
@@ -13171,7 +12206,9 @@
       <c r="I45" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J45" s="8"/>
+      <c r="J45" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K45" s="8" t="s">
         <v>52</v>
       </c>
@@ -13222,7 +12259,9 @@
       <c r="I46" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J46" s="8"/>
+      <c r="J46" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K46" s="8" t="s">
         <v>52</v>
       </c>
@@ -13272,7 +12311,9 @@
       <c r="I47" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="J47" s="8"/>
+      <c r="J47" s="8" t="s">
+        <v>92</v>
+      </c>
       <c r="K47" s="8" t="s">
         <v>52</v>
       </c>
@@ -13327,7 +12368,9 @@
       <c r="I48" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J48" s="8"/>
+      <c r="J48" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="K48" s="8" t="s">
         <v>52</v>
       </c>
@@ -13377,7 +12420,9 @@
       <c r="I49" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="J49" s="8"/>
+      <c r="J49" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="K49" s="8" t="s">
         <v>64</v>
       </c>
@@ -13433,7 +12478,9 @@
       <c r="I50" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J50" s="8"/>
+      <c r="J50" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="K50" s="8" t="s">
         <v>47</v>
       </c>
@@ -13484,7 +12531,9 @@
       <c r="I51" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J51" s="8"/>
+      <c r="J51" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="K51" s="8" t="s">
         <v>52</v>
       </c>
@@ -13536,7 +12585,9 @@
       <c r="I52" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="J52" s="8"/>
+      <c r="J52" s="8" t="s">
+        <v>90</v>
+      </c>
       <c r="K52" t="s">
         <v>52</v>
       </c>
@@ -21985,6 +21036,9 @@
       <c r="G2" t="s">
         <v>24</v>
       </c>
+      <c r="I2" t="s">
+        <v>75</v>
+      </c>
       <c r="O2">
         <f t="shared" ref="O2:O33" si="0">(INT(D2)*60+(D2-INT(D2))*100)-(INT($D$2)*60+($D$2-INT($D$2))*100)</f>
         <v>0</v>
@@ -22024,6 +21078,9 @@
       <c r="G3" t="s">
         <v>26</v>
       </c>
+      <c r="I3" t="s">
+        <v>75</v>
+      </c>
       <c r="O3">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -22063,6 +21120,9 @@
       <c r="G4" t="s">
         <v>28</v>
       </c>
+      <c r="I4" t="s">
+        <v>46</v>
+      </c>
       <c r="O4">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -22101,6 +21161,9 @@
       <c r="G5" t="s">
         <v>30</v>
       </c>
+      <c r="I5" t="s">
+        <v>46</v>
+      </c>
       <c r="O5">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -22139,6 +21202,9 @@
       <c r="G6" s="15" t="s">
         <v>32</v>
       </c>
+      <c r="I6" t="s">
+        <v>46</v>
+      </c>
       <c r="O6">
         <f t="shared" si="0"/>
         <v>4.9999999999990905</v>
@@ -22177,6 +21243,9 @@
       </c>
       <c r="G7" t="s">
         <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>75</v>
       </c>
       <c r="O7">
         <f t="shared" si="0"/>

</xml_diff>